<commit_message>
por fin sirve (gracias gabriel jajaj)
</commit_message>
<xml_diff>
--- a/Violencia Valle del Cauca Indices con Página con todo junto.xlsx
+++ b/Violencia Valle del Cauca Indices con Página con todo junto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juan Camilo Gómez\Desktop\universidad\Analítica Computacional\Módulo 1\Proyecto 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163BDB71-7574-41DF-9D96-2525BCDED7DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5597892-0796-4018-9E4C-F286D4DE4F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Habitantes" sheetId="49" r:id="rId1"/>

</xml_diff>